<commit_message>
Major update to arduino.html
</commit_message>
<xml_diff>
--- a/Voltage_discharge.xlsx
+++ b/Voltage_discharge.xlsx
@@ -606,7 +606,7 @@
           <c:x val="9.1001100000000015E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999831"/>
+          <c:h val="0.8103369999999982"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1879,11 +1879,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="129728896"/>
-        <c:axId val="129731968"/>
+        <c:axId val="169767296"/>
+        <c:axId val="169770368"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="129728896"/>
+        <c:axId val="169767296"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1915,14 +1915,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129731968"/>
+        <c:crossAx val="169770368"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="129731968"/>
+        <c:axId val="169770368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -1965,7 +1965,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129728896"/>
+        <c:crossAx val="169767296"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -1989,7 +1989,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000212E-2"/>
+          <c:h val="6.4066700000000226E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -2029,7 +2029,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000155" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000155" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000167" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000167" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -2049,7 +2049,7 @@
           <c:x val="9.1001100000000015E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999831"/>
+          <c:h val="0.8103369999999982"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -3488,11 +3488,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="129538304"/>
-        <c:axId val="129544192"/>
+        <c:axId val="169576704"/>
+        <c:axId val="169582592"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="129538304"/>
+        <c:axId val="169576704"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3524,14 +3524,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129544192"/>
+        <c:crossAx val="169582592"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="129544192"/>
+        <c:axId val="169582592"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -3574,7 +3574,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129538304"/>
+        <c:crossAx val="169576704"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -3598,7 +3598,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000212E-2"/>
+          <c:h val="6.4066700000000226E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -3638,7 +3638,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000155" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000155" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000167" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000167" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -3655,10 +3655,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="9.1082899999999994E-2"/>
+          <c:x val="9.1082900000000008E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89393599999999951"/>
-          <c:h val="0.81033699999999831"/>
+          <c:h val="0.8103369999999982"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -4600,11 +4600,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="129682816"/>
-        <c:axId val="129684608"/>
+        <c:axId val="169696640"/>
+        <c:axId val="169702528"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="129682816"/>
+        <c:axId val="169696640"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4636,14 +4636,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129684608"/>
+        <c:crossAx val="169702528"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="3"/>
         <c:minorUnit val="1.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="129684608"/>
+        <c:axId val="169702528"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -4685,7 +4685,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129682816"/>
+        <c:crossAx val="169696640"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -4709,7 +4709,7 @@
           <c:x val="7.5226400000000082E-2"/>
           <c:y val="0"/>
           <c:w val="0.88994100000000065"/>
-          <c:h val="6.4066700000000212E-2"/>
+          <c:h val="6.4066700000000226E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -4749,7 +4749,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000155" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000155" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000167" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000167" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -4769,7 +4769,7 @@
           <c:x val="9.1001100000000015E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.89403199999999949"/>
-          <c:h val="0.81033699999999831"/>
+          <c:h val="0.8103369999999982"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -6042,11 +6042,11 @@
             </c:numRef>
           </c:yVal>
         </c:ser>
-        <c:axId val="129725568"/>
-        <c:axId val="129727104"/>
+        <c:axId val="169755776"/>
+        <c:axId val="169757312"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="129725568"/>
+        <c:axId val="169755776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6078,14 +6078,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129727104"/>
+        <c:crossAx val="169757312"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
         <c:minorUnit val="0.5"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="129727104"/>
+        <c:axId val="169757312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13"/>
@@ -6128,7 +6128,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129725568"/>
+        <c:crossAx val="169755776"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -6188,7 +6188,7 @@
           <c:x val="7.5607700000000014E-2"/>
           <c:y val="0"/>
           <c:w val="0.88914199999999999"/>
-          <c:h val="6.4066700000000212E-2"/>
+          <c:h val="6.4066700000000226E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6232,7 +6232,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000155" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000155" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000167" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000167" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -6249,10 +6249,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="6.4312400000000297E-2"/>
+          <c:x val="6.4312400000000325E-2"/>
           <c:y val="0.12368000000000012"/>
           <c:w val="0.88765000000000005"/>
-          <c:h val="0.81033699999999831"/>
+          <c:h val="0.8103369999999982"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -6460,11 +6460,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="129903616"/>
-        <c:axId val="129909504"/>
+        <c:axId val="169815040"/>
+        <c:axId val="169816832"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="129903616"/>
+        <c:axId val="169815040"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="806395000"/>
@@ -6497,12 +6497,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129909504"/>
+        <c:crossAx val="169816832"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="129909504"/>
+        <c:axId val="169816832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6543,7 +6543,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="129903616"/>
+        <c:crossAx val="169815040"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.2"/>
@@ -6567,7 +6567,7 @@
           <c:x val="4.0081200000000004E-2"/>
           <c:y val="0"/>
           <c:w val="0.9"/>
-          <c:h val="6.4066700000000212E-2"/>
+          <c:h val="6.4066700000000226E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6607,7 +6607,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000155" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000155" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000167" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000167" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -6640,7 +6640,7 @@
                 <a:latin typeface="Arial" pitchFamily="34" charset="0"/>
                 <a:cs typeface="Arial" pitchFamily="34" charset="0"/>
               </a:rPr>
-              <a:t>Current Production</a:t>
+              <a:t>Current Generation</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0">
@@ -7245,11 +7245,11 @@
           </c:val>
         </c:ser>
         <c:marker val="1"/>
-        <c:axId val="130158976"/>
-        <c:axId val="130160512"/>
+        <c:axId val="170063360"/>
+        <c:axId val="170064896"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="130158976"/>
+        <c:axId val="170063360"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7273,14 +7273,14 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="130160512"/>
+        <c:crossAx val="170064896"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="130160512"/>
+        <c:axId val="170064896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7335,7 +7335,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="130158976"/>
+        <c:crossAx val="170063360"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7374,7 +7374,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75000000000000111" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000111" header="0.30000000000000032" footer="0.30000000000000032"/>
+    <c:pageMargins b="0.75000000000000122" l="0.70000000000000062" r="0.70000000000000062" t="0.75000000000000122" header="0.30000000000000032" footer="0.30000000000000032"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>

</xml_diff>